<commit_message>
update: documentations git push origin main
</commit_message>
<xml_diff>
--- a/FYP-ProgressTrack.xlsx
+++ b/FYP-ProgressTrack.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamlotfi/Desktop/FYP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3898C9E-C6E3-194C-AE7D-9D092AAF440E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16BB0049-549D-1E48-874D-9DD07F1E3E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{18A0949A-A941-4942-A929-12DEA1FC6C68}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="58">
   <si>
     <t>Task ID</t>
   </si>
@@ -207,6 +207,9 @@
   </si>
   <si>
     <t>https://docs.google.com/document/d/1rVbWoatZkmNisgtaDAgxFU5iTkoyqhf5CVGZ_pejgjM/edit?usp=sharing</t>
+  </si>
+  <si>
+    <t>DONE</t>
   </si>
 </sst>
 </file>
@@ -686,7 +689,9 @@
       <c r="E4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="F4" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G4" s="1"/>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.2">
@@ -702,7 +707,9 @@
       <c r="E5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="1"/>
+      <c r="F5" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.2">
@@ -718,7 +725,9 @@
       <c r="E6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="1"/>
+      <c r="F6" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.2">
@@ -734,7 +743,9 @@
       <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="1"/>
+      <c r="F7" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.2">
@@ -750,7 +761,9 @@
       <c r="E8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="1"/>
+      <c r="F8" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.2">
@@ -766,7 +779,9 @@
       <c r="E9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="1"/>
+      <c r="F9" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G9" s="1"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.2">
@@ -782,7 +797,9 @@
       <c r="E10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="1"/>
+      <c r="F10" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.2">
@@ -798,7 +815,9 @@
       <c r="E11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="1"/>
+      <c r="F11" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G11" s="1"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
@@ -814,7 +833,9 @@
       <c r="E12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F12" s="1"/>
+      <c r="F12" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="G12" s="1"/>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.2">

</xml_diff>